<commit_message>
Admin: edit data/showcase.xlsx via table editor
</commit_message>
<xml_diff>
--- a/data/showcase.xlsx
+++ b/data/showcase.xlsx
@@ -520,10 +520,10 @@
         <v>Ganpati 2026 — Aarti &amp; Documents</v>
       </c>
       <c r="B5" t="str">
-        <v>Ganpati Aarti Sheet (example)</v>
+        <v xml:space="preserve">Ganpati Aarti </v>
       </c>
       <c r="C5" t="str">
-        <v>Example row — replace DocumentURL with a real PDF, or delete this row.</v>
+        <v xml:space="preserve">Sankalp Ganpati Aarti </v>
       </c>
       <c r="D5" t="str">
         <v>Documents</v>
@@ -535,13 +535,13 @@
         <v/>
       </c>
       <c r="G5" t="str">
-        <v>docs/showcase/replace-with-your-aarti.pdf</v>
+        <v>docs/showcase/Sankalp Aarati Sangraha 2023</v>
       </c>
       <c r="H5" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="I5" t="str">
-        <v>100</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">

</xml_diff>